<commit_message>
Document role links for HSQ app
</commit_message>
<xml_diff>
--- a/base/Base_HSQ_Admin.xlsx
+++ b/base/Base_HSQ_Admin.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="R854a8ef6ae2445bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuracion" sheetId="2" r:id="R77f22551ec144f38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz_Activos" sheetId="3" r:id="R6e6f0b2b720642d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyectos" sheetId="4" r:id="R14bd505fc2c74dbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formularios" sheetId="5" r:id="R388d029356944e10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preguntas" sheetId="6" r:id="Reff7dd2ff6164d16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opciones" sheetId="7" r:id="R9dd7ec65ddae455b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tipos_Campo" sheetId="8" r:id="Rc3ced4da89d34675"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exportador_Config" sheetId="9" r:id="R1d456d71fcea4387"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Respuestas_Ejemplo" sheetId="10" r:id="R7afce0afc2a148d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="Rbeadd3bc97ab4696"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuracion" sheetId="2" r:id="Rca09970462ce4a16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz_Activos" sheetId="3" r:id="Rc3e863afa1f3434b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyectos" sheetId="4" r:id="R9342d657a14d4f8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formularios" sheetId="5" r:id="Rfdef8f7d86cd436e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preguntas" sheetId="6" r:id="Re504655b5c8a4a07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opciones" sheetId="7" r:id="R75094dd08cd34259"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tipos_Campo" sheetId="8" r:id="R709e4c8c86484c86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exportador_Config" sheetId="9" r:id="Re4e7085488354b2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Respuestas_Ejemplo" sheetId="10" r:id="Rf9e435b81e084744"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -251,8 +251,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabla_Configuracion" displayName="Tabla_Configuracion" ref="A1:C7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:C7"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tabla_Configuracion" displayName="Tabla_Configuracion" ref="A1:C8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:C8"/>
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="parametro"/>
     <x:tableColumn id="2" name="valor"/>
@@ -640,7 +640,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3a6ec4bcaad4b00"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae0c384667f14d22"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -707,10 +707,10 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="13" t="n">
-        <x:v>46218.72972940972</x:v>
+        <x:v>46218.741428877314</x:v>
       </x:c>
       <x:c r="B2" s="20" t="n">
-        <x:v>46218.72972940972</x:v>
+        <x:v>46218.741428877314</x:v>
       </x:c>
       <x:c r="C2" s="20" t="str">
         <x:v>PREOPERACIONAL-20260715-000001</x:v>
@@ -747,7 +747,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1da47ff89a5446fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R466ce794cdb14cd0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -757,7 +757,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18.25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="97.62999725341797" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="51.880001068115234" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -828,20 +828,31 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="13" t="str">
+      <x:c r="A7" s="11" t="str">
         <x:v>PREGUNTAS_PROMEDIO_FORMULARIO</x:v>
       </x:c>
-      <x:c r="B7" s="20" t="n">
+      <x:c r="B7" s="19" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C7" s="14" t="str">
+      <x:c r="C7" s="12" t="str">
         <x:v>Cantidad promedio indicada por HSQ.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="13" t="str">
+        <x:v>WEB_APP_URL</x:v>
+      </x:c>
+      <x:c r="B8" s="20" t="str">
+        <x:v>https://script.google.com/macros/s/AKfycbyDhvIfqO6kY4uwqL4aiTLEZe2pdaiV-mFwpZ3ytzV5TjQvJUhrPMSNoJtPNT948pYl7w/exec</x:v>
+      </x:c>
+      <x:c r="C8" s="14" t="str">
+        <x:v>URL oficial que usan mensajeros, coordinadores y HSQ.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d20fa6640a04957"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb78058ce122344d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43549,7 +43560,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5473b1c74e64262"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbddd565a498144ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45117,7 +45128,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9198d82aee984759"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6f612b81e1f46a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45202,7 +45213,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R639ce15184134c93"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64bbf020f8734cbf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46147,7 +46158,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ad6da7694554847"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9ad4c93848b4df6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46417,7 +46428,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f5fd232c4da4901"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f5a1b69d4034ddf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46575,7 +46586,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65eb4b2b9fd24d72"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0c3e9bd118f4536"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46658,7 +46669,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1efcdf0f4aa421f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd026056e9efa4959"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>